<commit_message>
Physical parameters from global to specific to alloy
</commit_message>
<xml_diff>
--- a/V4_without_z1.xlsx
+++ b/V4_without_z1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DE\sem 5\Codes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53D3E9C9-5A81-4C3F-ADB4-6B5676AE50AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9F6A336-B0A3-4334-BF25-B06B52CF10AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-756" windowWidth="23256" windowHeight="12576" xr2:uid="{7DCB483B-EADE-468B-A11D-0B02376EF2F9}"/>
   </bookViews>
@@ -17419,13 +17419,13 @@
         <v>5.5399999999999998E-2</v>
       </c>
       <c r="O246" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P246" s="7">
         <v>0</v>
       </c>
       <c r="Q246" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R246" s="5">
         <v>121476</v>

</xml_diff>